<commit_message>
update with sa initialization
</commit_message>
<xml_diff>
--- a/data/data-23-24.xlsx
+++ b/data/data-23-24.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9144" firstSheet="2" activeTab="3"/>
+    <workbookView windowWidth="22188" windowHeight="9144" firstSheet="2" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="classroomLt" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="126">
   <si>
     <t>ID</t>
   </si>
@@ -126,13 +126,223 @@
     <t>Data Warehouse</t>
   </si>
   <si>
+    <t>214362-01-01</t>
+  </si>
+  <si>
+    <t>Giao tiếp người-máy</t>
+  </si>
+  <si>
+    <t>DH21DT</t>
+  </si>
+  <si>
+    <t>214362-03-01</t>
+  </si>
+  <si>
+    <t>214362-512-01</t>
+  </si>
+  <si>
+    <t>214362-02-01</t>
+  </si>
+  <si>
+    <t>214451-01</t>
+  </si>
+  <si>
+    <t>Hệ quản trị cơ sở dữ liệu</t>
+  </si>
+  <si>
+    <t>214451-04</t>
+  </si>
+  <si>
+    <t>214451-03</t>
+  </si>
+  <si>
+    <t>214372-01</t>
+  </si>
+  <si>
+    <t>Lập trình .NET</t>
+  </si>
+  <si>
+    <t>214321-03</t>
+  </si>
+  <si>
+    <t>Lập trình cơ bản</t>
+  </si>
+  <si>
+    <t>214321-01</t>
+  </si>
+  <si>
+    <t>214321-505</t>
+  </si>
+  <si>
+    <t>DH20DT</t>
+  </si>
+  <si>
+    <t>214321-02</t>
+  </si>
+  <si>
+    <t>214252-02</t>
+  </si>
+  <si>
+    <t>Lập trình mạng</t>
+  </si>
+  <si>
+    <t>214252-03</t>
+  </si>
+  <si>
+    <t>214252-04</t>
+  </si>
+  <si>
+    <t>214252-01</t>
+  </si>
+  <si>
+    <t>214462-04-01</t>
+  </si>
+  <si>
+    <t>Lập trình Web</t>
+  </si>
+  <si>
+    <t>214462-02-02</t>
+  </si>
+  <si>
+    <t>214462-01-03</t>
+  </si>
+  <si>
+    <t>214462-03-04</t>
+  </si>
+  <si>
+    <t>214241-512</t>
+  </si>
+  <si>
+    <t>Mạng máy tính cơ bản</t>
+  </si>
+  <si>
+    <t>214282-01</t>
+  </si>
+  <si>
+    <t>Mạng máy tính nâng cao</t>
+  </si>
+  <si>
+    <t>214201-01</t>
+  </si>
+  <si>
+    <t>Nhập môn tin học</t>
+  </si>
+  <si>
+    <t>214201-02</t>
+  </si>
+  <si>
+    <t>214201-505</t>
+  </si>
+  <si>
+    <t>214201-03</t>
+  </si>
+  <si>
+    <t>214463-01</t>
+  </si>
+  <si>
+    <t>Nhập môn trí tuệ nhân tạo</t>
+  </si>
+  <si>
+    <t>214463-03</t>
+  </si>
+  <si>
+    <t>214463-02</t>
+  </si>
+  <si>
+    <t>214463-04</t>
+  </si>
+  <si>
+    <t>214383-01</t>
+  </si>
+  <si>
+    <t>Quản lý dự án phần mềm</t>
+  </si>
+  <si>
+    <t>214389-03</t>
+  </si>
+  <si>
+    <t>Toán rời rạc</t>
+  </si>
+  <si>
+    <t>214389-02</t>
+  </si>
+  <si>
+    <t>214389-01</t>
+  </si>
+  <si>
+    <t>DH22DT</t>
+  </si>
+  <si>
+    <t>Subject id</t>
+  </si>
+  <si>
+    <t>Credit</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Exam time</t>
+  </si>
+  <si>
+    <t>Lesson time</t>
+  </si>
+  <si>
+    <t>214201</t>
+  </si>
+  <si>
+    <t>214241</t>
+  </si>
+  <si>
+    <t>214252</t>
+  </si>
+  <si>
+    <t>214282</t>
+  </si>
+  <si>
+    <t>214321</t>
+  </si>
+  <si>
     <t>214362-01</t>
   </si>
   <si>
-    <t>Giao tiếp người-máy</t>
-  </si>
-  <si>
-    <t>DH21DT</t>
+    <t>Giao tiếp người _máy</t>
+  </si>
+  <si>
+    <t>214372</t>
+  </si>
+  <si>
+    <t>214379</t>
+  </si>
+  <si>
+    <t>214383</t>
+  </si>
+  <si>
+    <t>214389</t>
+  </si>
+  <si>
+    <t>214441</t>
+  </si>
+  <si>
+    <t>214451</t>
+  </si>
+  <si>
+    <t>214462-01</t>
+  </si>
+  <si>
+    <t>214463</t>
+  </si>
+  <si>
+    <t>214464</t>
+  </si>
+  <si>
+    <t>214485</t>
+  </si>
+  <si>
+    <t>214491</t>
+  </si>
+  <si>
+    <t>214362-02</t>
   </si>
   <si>
     <t>214362-03</t>
@@ -141,187 +351,46 @@
     <t>214362-512</t>
   </si>
   <si>
-    <t>214362-02</t>
-  </si>
-  <si>
-    <t>214451-01</t>
-  </si>
-  <si>
-    <t>Hệ quản trị cơ sở dữ liệu</t>
-  </si>
-  <si>
-    <t>214451-04</t>
-  </si>
-  <si>
-    <t>214451-03</t>
-  </si>
-  <si>
-    <t>214372-01</t>
-  </si>
-  <si>
-    <t>Lập trình .NET</t>
-  </si>
-  <si>
-    <t>214321-03</t>
-  </si>
-  <si>
-    <t>Lập trình cơ bản</t>
-  </si>
-  <si>
-    <t>214321-01</t>
-  </si>
-  <si>
-    <t>214321-505</t>
-  </si>
-  <si>
-    <t>DH20DT</t>
-  </si>
-  <si>
-    <t>214321-02</t>
-  </si>
-  <si>
-    <t>214252-02</t>
-  </si>
-  <si>
-    <t>Lập trình mạng</t>
-  </si>
-  <si>
-    <t>214252-03</t>
-  </si>
-  <si>
-    <t>214252-04</t>
-  </si>
-  <si>
-    <t>214252-01</t>
+    <t>214462-02</t>
+  </si>
+  <si>
+    <t>214462-03</t>
   </si>
   <si>
     <t>214462-04</t>
   </si>
   <si>
-    <t>Lập trình Web</t>
-  </si>
-  <si>
-    <t>214462-02</t>
-  </si>
-  <si>
-    <t>214462-01</t>
-  </si>
-  <si>
-    <t>214462-03</t>
-  </si>
-  <si>
-    <t>214241-512</t>
-  </si>
-  <si>
-    <t>Mạng máy tính cơ bản</t>
-  </si>
-  <si>
-    <t>214282-01</t>
-  </si>
-  <si>
-    <t>Mạng máy tính nâng cao</t>
-  </si>
-  <si>
-    <t>214201-01</t>
-  </si>
-  <si>
-    <t>Nhập môn tin học</t>
-  </si>
-  <si>
-    <t>214201-02</t>
-  </si>
-  <si>
-    <t>214201-505</t>
-  </si>
-  <si>
-    <t>214201-03</t>
-  </si>
-  <si>
-    <t>214463-01</t>
-  </si>
-  <si>
-    <t>Nhập môn trí tuệ nhân tạo</t>
-  </si>
-  <si>
-    <t>214463-03</t>
-  </si>
-  <si>
-    <t>214463-02</t>
-  </si>
-  <si>
-    <t>214463-04</t>
-  </si>
-  <si>
-    <t>214383-01</t>
-  </si>
-  <si>
-    <t>Quản lý dự án phần mềm</t>
-  </si>
-  <si>
-    <t>214389-03</t>
-  </si>
-  <si>
-    <t>Toán rời rạc</t>
-  </si>
-  <si>
-    <t>214389-02</t>
-  </si>
-  <si>
-    <t>214389-01</t>
-  </si>
-  <si>
-    <t>DH22DT</t>
-  </si>
-  <si>
-    <t>Subject id</t>
-  </si>
-  <si>
-    <t>Credit</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Exam time</t>
-  </si>
-  <si>
-    <t>Lesson time</t>
-  </si>
-  <si>
-    <t>Giao tiếp người _máy</t>
-  </si>
-  <si>
     <t>Exam date</t>
   </si>
   <si>
-    <t>2022-10-12</t>
-  </si>
-  <si>
-    <t>2022-10-13</t>
-  </si>
-  <si>
-    <t>2022-10-14</t>
-  </si>
-  <si>
-    <t>2022-10-15</t>
-  </si>
-  <si>
-    <t>2022-10-16</t>
-  </si>
-  <si>
-    <t>2022-10-17</t>
-  </si>
-  <si>
-    <t>2022-10-18</t>
-  </si>
-  <si>
-    <t>2022-10-19</t>
-  </si>
-  <si>
-    <t>2022-10-20</t>
-  </si>
-  <si>
-    <t>2022-10-21</t>
+    <t>2024-01-08</t>
+  </si>
+  <si>
+    <t>2024-01-09</t>
+  </si>
+  <si>
+    <t>2024-01-10</t>
+  </si>
+  <si>
+    <t>2024-01-11</t>
+  </si>
+  <si>
+    <t>2024-01-12</t>
+  </si>
+  <si>
+    <t>2024-01-15</t>
+  </si>
+  <si>
+    <t>2024-01-16</t>
+  </si>
+  <si>
+    <t>2024-01-17</t>
+  </si>
+  <si>
+    <t>2024-01-18</t>
+  </si>
+  <si>
+    <t>2024-01-19</t>
   </si>
   <si>
     <t>Academy year</t>
@@ -978,17 +1047,20 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1"/>
@@ -1587,12 +1659,12 @@
   <cols>
     <col min="1" max="1" width="15.8888888888889" customWidth="1"/>
     <col min="2" max="2" width="40.5555555555556" customWidth="1"/>
-    <col min="3" max="3" width="17.4444444444444" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.4444444444444" style="3" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="11.6666666666667" style="2" customWidth="1"/>
+    <col min="5" max="5" width="11.6666666666667" style="3" customWidth="1"/>
     <col min="6" max="6" width="3.66666666666667" customWidth="1"/>
-    <col min="7" max="7" width="10.7777777777778" style="2" customWidth="1"/>
-    <col min="8" max="8" width="8.88888888888889" style="8"/>
+    <col min="7" max="7" width="10.7777777777778" style="3" customWidth="1"/>
+    <col min="8" max="8" width="8.88888888888889" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1602,985 +1674,985 @@
       <c r="B1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D1" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>19</v>
       </c>
       <c r="F1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="10">
         <v>123</v>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="11">
         <v>123</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>12</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="11">
         <v>12</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F3">
         <v>2</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <v>112</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="11">
         <v>112</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F4">
         <v>3</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="10">
         <v>115</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="11">
         <v>115</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F5">
         <v>4</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="10">
         <v>110</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="11">
         <v>110</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F6">
         <v>5</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="10">
         <v>150</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="11">
         <v>150</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F7">
         <v>6</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:7">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="10">
         <v>122</v>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="11">
         <v>122</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F8">
         <v>7</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="10">
         <v>121</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="11">
         <v>121</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F9">
         <v>8</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="10">
         <v>106</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="11">
         <v>106</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F10">
         <v>9</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="10">
         <v>95</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="11">
         <v>95</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F11">
         <v>10</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="10">
         <v>12</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="11">
         <v>12</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F12">
         <v>11</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="10">
         <v>105</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="11">
         <v>105</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F13">
         <v>12</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="10">
         <v>109</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="11">
         <v>109</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F14">
         <v>13</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="10">
         <v>108</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="11">
         <v>108</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F15">
         <v>14</v>
       </c>
-      <c r="G15" s="2">
+      <c r="G15" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="10">
         <v>112</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="11">
         <v>112</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F16">
         <v>15</v>
       </c>
-      <c r="G16" s="2">
+      <c r="G16" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="10">
         <v>123</v>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="11">
         <v>123</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F17">
         <v>16</v>
       </c>
-      <c r="G17" s="2">
+      <c r="G17" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="10">
         <v>151</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="11">
         <v>151</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F18">
         <v>17</v>
       </c>
-      <c r="G18" s="2">
+      <c r="G18" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="10">
         <v>107</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="11">
         <v>107</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F19">
         <v>18</v>
       </c>
-      <c r="G19" s="2">
+      <c r="G19" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="10">
         <v>15</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="11">
         <v>15</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F20">
         <v>19</v>
       </c>
-      <c r="G20" s="2">
+      <c r="G20" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="9">
+      <c r="C21" s="10">
         <v>110</v>
       </c>
-      <c r="D21" s="10">
+      <c r="D21" s="11">
         <v>110</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F21">
         <v>20</v>
       </c>
-      <c r="G21" s="2">
+      <c r="G21" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C22" s="9">
+      <c r="C22" s="10">
         <v>110</v>
       </c>
-      <c r="D22" s="10">
+      <c r="D22" s="11">
         <v>110</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F22">
         <v>21</v>
       </c>
-      <c r="G22" s="2">
+      <c r="G22" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="9">
+      <c r="C23" s="10">
         <v>114</v>
       </c>
-      <c r="D23" s="10">
+      <c r="D23" s="11">
         <v>114</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F23">
         <v>22</v>
       </c>
-      <c r="G23" s="2">
+      <c r="G23" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="10">
         <v>111</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="11">
         <v>111</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F24">
         <v>23</v>
       </c>
-      <c r="G24" s="2">
+      <c r="G24" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C25" s="9">
+      <c r="C25" s="10">
         <v>110</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="11">
         <v>110</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F25">
         <v>24</v>
       </c>
-      <c r="G25" s="2">
+      <c r="G25" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" spans="1:7">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="9">
+      <c r="C26" s="10">
         <v>111</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="11">
         <v>111</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F26">
         <v>25</v>
       </c>
-      <c r="G26" s="2">
+      <c r="G26" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:7">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="10">
         <v>110</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="11">
         <v>110</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F27">
         <v>26</v>
       </c>
-      <c r="G27" s="2">
+      <c r="G27" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1" spans="1:7">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28" s="10">
         <v>105</v>
       </c>
-      <c r="D28" s="10">
+      <c r="D28" s="11">
         <v>105</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F28">
         <v>27</v>
       </c>
-      <c r="G28" s="2">
+      <c r="G28" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:7">
-      <c r="A29" s="8" t="s">
+      <c r="A29" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29" s="10">
         <v>109</v>
       </c>
-      <c r="D29" s="10">
+      <c r="D29" s="11">
         <v>109</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="E29" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F29">
         <v>28</v>
       </c>
-      <c r="G29" s="2">
+      <c r="G29" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:7">
-      <c r="A30" s="8" t="s">
+      <c r="A30" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="9">
+      <c r="C30" s="10">
         <v>12</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="11">
         <v>12</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E30" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F30">
         <v>29</v>
       </c>
-      <c r="G30" s="2">
+      <c r="G30" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:7">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C31" s="9">
+      <c r="C31" s="10">
         <v>101</v>
       </c>
-      <c r="D31" s="10">
+      <c r="D31" s="11">
         <v>101</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="E31" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F31">
         <v>30</v>
       </c>
-      <c r="G31" s="2">
+      <c r="G31" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="32" spans="1:7">
-      <c r="A32" s="8" t="s">
+      <c r="A32" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C32" s="9">
+      <c r="C32" s="10">
         <v>135</v>
       </c>
-      <c r="D32" s="10">
+      <c r="D32" s="11">
         <v>135</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E32" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F32">
         <v>31</v>
       </c>
-      <c r="G32" s="2">
+      <c r="G32" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:7">
-      <c r="A33" s="8" t="s">
+      <c r="A33" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C33" s="9">
+      <c r="C33" s="10">
         <v>113</v>
       </c>
-      <c r="D33" s="10">
+      <c r="D33" s="11">
         <v>113</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F33">
         <v>32</v>
       </c>
-      <c r="G33" s="2">
+      <c r="G33" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="34" spans="1:7">
-      <c r="A34" s="8" t="s">
+      <c r="A34" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C34" s="9">
+      <c r="C34" s="10">
         <v>15</v>
       </c>
-      <c r="D34" s="10">
+      <c r="D34" s="11">
         <v>15</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="E34" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F34">
         <v>33</v>
       </c>
-      <c r="G34" s="2">
+      <c r="G34" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="35" spans="1:7">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C35" s="9">
+      <c r="C35" s="10">
         <v>122</v>
       </c>
-      <c r="D35" s="10">
+      <c r="D35" s="11">
         <v>122</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="E35" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F35">
         <v>34</v>
       </c>
-      <c r="G35" s="2">
+      <c r="G35" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="36" spans="1:7">
-      <c r="A36" s="8" t="s">
+      <c r="A36" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C36" s="9">
+      <c r="C36" s="10">
         <v>90</v>
       </c>
-      <c r="D36" s="10">
+      <c r="D36" s="11">
         <v>90</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="E36" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F36">
         <v>35</v>
       </c>
-      <c r="G36" s="2">
+      <c r="G36" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="37" spans="1:7">
-      <c r="A37" s="8" t="s">
+      <c r="A37" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="B37" s="8" t="s">
+      <c r="B37" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="10">
         <v>94</v>
       </c>
-      <c r="D37" s="10">
+      <c r="D37" s="11">
         <v>94</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="E37" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F37">
         <v>36</v>
       </c>
-      <c r="G37" s="2">
+      <c r="G37" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="38" spans="1:7">
-      <c r="A38" s="8" t="s">
+      <c r="A38" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="10">
         <v>92</v>
       </c>
-      <c r="D38" s="10">
+      <c r="D38" s="11">
         <v>92</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="E38" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F38">
         <v>37</v>
       </c>
-      <c r="G38" s="2">
+      <c r="G38" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="39" spans="1:7">
-      <c r="A39" s="8" t="s">
+      <c r="A39" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B39" s="8" t="s">
+      <c r="B39" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C39" s="9">
+      <c r="C39" s="10">
         <v>105</v>
       </c>
-      <c r="D39" s="10">
+      <c r="D39" s="11">
         <v>105</v>
       </c>
-      <c r="E39" s="2" t="s">
+      <c r="E39" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F39">
         <v>38</v>
       </c>
-      <c r="G39" s="2">
+      <c r="G39" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="40" spans="1:7">
-      <c r="A40" s="8" t="s">
+      <c r="A40" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C40" s="9">
+      <c r="C40" s="10">
         <v>46</v>
       </c>
-      <c r="D40" s="10">
+      <c r="D40" s="11">
         <v>46</v>
       </c>
-      <c r="E40" s="2" t="s">
+      <c r="E40" s="3" t="s">
         <v>23</v>
       </c>
       <c r="F40">
         <v>39</v>
       </c>
-      <c r="G40" s="2">
+      <c r="G40" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="41" spans="1:7">
-      <c r="A41" s="8" t="s">
+      <c r="A41" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B41" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="9">
+      <c r="C41" s="10">
         <v>105</v>
       </c>
-      <c r="D41" s="10">
+      <c r="D41" s="11">
         <v>105</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="E41" s="3" t="s">
         <v>51</v>
       </c>
       <c r="F41">
         <v>40</v>
       </c>
-      <c r="G41" s="2">
+      <c r="G41" s="3">
         <v>6</v>
       </c>
     </row>
     <row r="42" spans="1:7">
-      <c r="A42" s="8" t="s">
+      <c r="A42" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="B42" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C42" s="9">
+      <c r="C42" s="10">
         <v>105</v>
       </c>
-      <c r="D42" s="10">
+      <c r="D42" s="11">
         <v>105</v>
       </c>
-      <c r="E42" s="2" t="s">
+      <c r="E42" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F42">
         <v>41</v>
       </c>
-      <c r="G42" s="2">
+      <c r="G42" s="3">
         <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:7">
-      <c r="A43" s="8" t="s">
+      <c r="A43" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="B43" s="8" t="s">
+      <c r="B43" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C43" s="9">
+      <c r="C43" s="10">
         <v>106</v>
       </c>
-      <c r="D43" s="10">
+      <c r="D43" s="11">
         <v>106</v>
       </c>
-      <c r="E43" s="2" t="s">
+      <c r="E43" s="3" t="s">
         <v>83</v>
       </c>
       <c r="F43">
         <v>42</v>
       </c>
-      <c r="G43" s="2">
+      <c r="G43" s="3">
         <v>8</v>
       </c>
     </row>
@@ -7075,15 +7147,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="11.8888888888889" style="1"/>
+    <col min="1" max="1" width="11.8888888888889" style="2"/>
     <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="8.88888888888889" style="2"/>
+    <col min="3" max="3" width="8.88888888888889" style="3"/>
     <col min="4" max="4" width="5.55555555555556" customWidth="1"/>
     <col min="5" max="5" width="10.1111111111111" customWidth="1"/>
-    <col min="6" max="6" width="10.8888888888889" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.8888888888889" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -7093,7 +7165,7 @@
       <c r="B1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>85</v>
       </c>
       <c r="D1" t="s">
@@ -7102,347 +7174,467 @@
       <c r="E1" t="s">
         <v>87</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="2" ht="15.6" spans="1:6">
-      <c r="A2" s="3">
-        <v>214201</v>
-      </c>
-      <c r="B2" s="4" t="s">
+      <c r="A2" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="6">
         <v>0</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="7">
         <v>1</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="7">
         <v>2</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="3" ht="15.6" spans="1:6">
-      <c r="A3" s="3">
-        <v>214241</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="A3" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="6">
         <v>0</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="7">
         <v>0</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="7">
         <v>2</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="4" ht="15.6" spans="1:6">
-      <c r="A4" s="3">
-        <v>214252</v>
-      </c>
-      <c r="B4" s="4" t="s">
+      <c r="A4" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>0</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="7">
         <v>1</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="7">
         <v>2</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="5" ht="15.6" spans="1:6">
-      <c r="A5" s="3">
-        <v>214282</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="A5" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="6">
         <v>0</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="7">
         <v>0</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="7">
         <v>2</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="6" ht="15.6" spans="1:6">
-      <c r="A6" s="3">
-        <v>214321</v>
-      </c>
-      <c r="B6" s="4" t="s">
+      <c r="A6" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="6">
         <v>0</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="7">
         <v>1</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="7">
         <v>2</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="7" ht="15.6" spans="1:6">
-      <c r="A7" s="3">
-        <v>214362</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C7" s="5">
+      <c r="A7" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="6">
         <v>0</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="7">
         <v>2</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="7">
         <v>6</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="8" ht="15.6" spans="1:6">
-      <c r="A8" s="3">
-        <v>214372</v>
-      </c>
-      <c r="B8" s="4" t="s">
+      <c r="A8" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="6">
         <v>0</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="7">
         <v>2</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="7">
         <v>6</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="9" ht="15.6" spans="1:6">
-      <c r="A9" s="3">
-        <v>214379</v>
-      </c>
-      <c r="B9" s="4" t="s">
+      <c r="A9" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="6">
         <v>0</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="7">
         <v>2</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="7">
         <v>6</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="10" ht="15.6" spans="1:6">
-      <c r="A10" s="3">
-        <v>214383</v>
-      </c>
-      <c r="B10" s="4" t="s">
+      <c r="A10" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="6">
         <v>0</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="7">
         <v>0</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="7">
         <v>2</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="11" ht="15.6" spans="1:6">
-      <c r="A11" s="3">
-        <v>214389</v>
-      </c>
-      <c r="B11" s="4" t="s">
+      <c r="A11" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="6">
         <v>0</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="7">
         <v>0</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="7">
         <v>2</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="12" ht="15.6" spans="1:6">
-      <c r="A12" s="3">
-        <v>214441</v>
-      </c>
-      <c r="B12" s="4" t="s">
+      <c r="A12" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="6">
         <v>0</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="7">
         <v>0</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="7">
         <v>2</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F12" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="13" ht="15.6" spans="1:6">
-      <c r="A13" s="3">
-        <v>214451</v>
-      </c>
-      <c r="B13" s="4" t="s">
+      <c r="A13" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="6">
         <v>0</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="7">
         <v>0</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="7">
         <v>2</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="14" ht="15.6" spans="1:6">
-      <c r="A14" s="3">
-        <v>214462</v>
-      </c>
-      <c r="B14" s="4" t="s">
+      <c r="A14" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="6">
         <v>0</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="7">
         <v>2</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="7">
         <v>6</v>
       </c>
-      <c r="F14" s="7">
+      <c r="F14" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="15" ht="15.6" spans="1:6">
-      <c r="A15" s="3">
-        <v>214463</v>
-      </c>
-      <c r="B15" s="4" t="s">
+      <c r="A15" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="6">
         <v>0</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="7">
         <v>0</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="7">
         <v>2</v>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="16" ht="15.6" spans="1:6">
-      <c r="A16" s="3">
-        <v>214464</v>
-      </c>
-      <c r="B16" s="4" t="s">
+      <c r="A16" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="6">
         <v>0</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="7">
         <v>0</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="7">
         <v>2</v>
       </c>
-      <c r="F16" s="7">
+      <c r="F16" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="17" ht="15.6" spans="1:6">
-      <c r="A17" s="3">
-        <v>214485</v>
-      </c>
-      <c r="B17" s="4" t="s">
+      <c r="A17" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="6">
         <v>0</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="7">
         <v>0</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="7">
         <v>2</v>
       </c>
-      <c r="F17" s="7">
+      <c r="F17" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="18" ht="15.6" spans="1:6">
-      <c r="A18" s="3">
-        <v>214491</v>
-      </c>
-      <c r="B18" s="4" t="s">
+      <c r="A18" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="6">
         <v>0</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="7">
         <v>0</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="7">
         <v>2</v>
       </c>
-      <c r="F18" s="7">
+      <c r="F18" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" ht="15.6" spans="1:6">
+      <c r="A19" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0</v>
+      </c>
+      <c r="D19" s="7">
+        <v>2</v>
+      </c>
+      <c r="E19" s="7">
+        <v>6</v>
+      </c>
+      <c r="F19" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" ht="15.6" spans="1:6">
+      <c r="A20" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0</v>
+      </c>
+      <c r="D20" s="7">
+        <v>2</v>
+      </c>
+      <c r="E20" s="7">
+        <v>6</v>
+      </c>
+      <c r="F20" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" ht="15.6" spans="1:6">
+      <c r="A21" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C21" s="6">
+        <v>0</v>
+      </c>
+      <c r="D21" s="7">
+        <v>2</v>
+      </c>
+      <c r="E21" s="7">
+        <v>6</v>
+      </c>
+      <c r="F21" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" ht="15.6" spans="1:6">
+      <c r="A22" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="6">
+        <v>0</v>
+      </c>
+      <c r="D22" s="7">
+        <v>2</v>
+      </c>
+      <c r="E22" s="7">
+        <v>6</v>
+      </c>
+      <c r="F22" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" ht="15.6" spans="1:6">
+      <c r="A23" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0</v>
+      </c>
+      <c r="D23" s="7">
+        <v>2</v>
+      </c>
+      <c r="E23" s="7">
+        <v>6</v>
+      </c>
+      <c r="F23" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" ht="15.6" spans="1:6">
+      <c r="A24" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" s="6">
+        <v>0</v>
+      </c>
+      <c r="D24" s="7">
+        <v>2</v>
+      </c>
+      <c r="E24" s="7">
+        <v>6</v>
+      </c>
+      <c r="F24" s="8">
         <v>3</v>
       </c>
     </row>
@@ -7463,57 +7655,57 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="1" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="1" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="1" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="1" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="1" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="1" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="1" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="1" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -7533,10 +7725,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="B1" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" spans="1:2">

</xml_diff>